<commit_message>
added nr. of total re-draws; added which participants deviate most from benchmark; updated codebook
</commit_message>
<xml_diff>
--- a/results/codebooks/codebook_sim_results.xlsx
+++ b/results/codebooks/codebook_sim_results.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24334"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6341B324-917D-4663-8428-474D0B9984B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C6B629C1-56EE-40A9-91C6-125053890D69}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="64">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="76" uniqueCount="75">
   <si>
     <t>Variable Name</t>
   </si>
@@ -219,6 +219,39 @@
   </si>
   <si>
     <t>number of negative estimation problems (ICCs &lt;= -1/[k-1])</t>
+  </si>
+  <si>
+    <t>id_min_diff_ICC</t>
+  </si>
+  <si>
+    <t>ID of participant with the highest negative deviation between comparison ICC and benchmark ICC (i.e., minimum difference)</t>
+  </si>
+  <si>
+    <t>id_max_diff_ICC</t>
+  </si>
+  <si>
+    <t>ID of participant with the highest positive deviation between comparison ICC and benchmark ICC (i.e., maximum difference)</t>
+  </si>
+  <si>
+    <t>id_min_diff_ICC.z</t>
+  </si>
+  <si>
+    <t>id_max_diff_ICC.z</t>
+  </si>
+  <si>
+    <t>ID of participant with the highest negative deviation between comparison ICC (Fisher's Z-transformed) and benchmark ICC (Fisher's Z-transformed) (i.e., minimum difference)</t>
+  </si>
+  <si>
+    <t>ID of participant with the highest positive deviation between comparison ICC (Fisher's Z-transformed) and benchmark ICC (Fisher's Z-transformed) (i.e., maximum difference)</t>
+  </si>
+  <si>
+    <t>total_redraws</t>
+  </si>
+  <si>
+    <t xml:space="preserve">total number of re-draws of measurement occasions across participants per replications due to zero variance in initial draw </t>
+  </si>
+  <si>
+    <t>always 0 for ordered draws (did not occur in these conditions)</t>
   </si>
 </sst>
 </file>
@@ -575,7 +608,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D27"/>
+  <dimension ref="A1:D32"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="18.42578125" style="1" bestFit="1" customWidth="1"/>
@@ -702,147 +735,194 @@
       </c>
       <c r="C12" s="2"/>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="B13" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="C13" s="2"/>
+    </row>
+    <row r="14" spans="1:4" ht="45" x14ac:dyDescent="0.25">
+      <c r="A14" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="B14" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="C14" s="2"/>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A15" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="B13" s="1" t="s">
+      <c r="B15" s="1" t="s">
         <v>45</v>
-      </c>
-      <c r="C13" s="2"/>
-    </row>
-    <row r="14" spans="1:4" ht="60" x14ac:dyDescent="0.25">
-      <c r="A14" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="B14" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="C14" s="2"/>
-    </row>
-    <row r="15" spans="1:4" ht="60" x14ac:dyDescent="0.25">
-      <c r="A15" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="B15" s="1" t="s">
-        <v>47</v>
       </c>
       <c r="C15" s="2"/>
     </row>
     <row r="16" spans="1:4" ht="60" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="B16" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="C16" s="2"/>
+    </row>
+    <row r="17" spans="1:4" ht="60" x14ac:dyDescent="0.25">
+      <c r="A17" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="B17" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="C17" s="2"/>
+    </row>
+    <row r="18" spans="1:4" ht="60" x14ac:dyDescent="0.25">
+      <c r="A18" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="B16" s="1" t="s">
+      <c r="B18" s="1" t="s">
         <v>48</v>
-      </c>
-      <c r="C16" s="2"/>
-    </row>
-    <row r="17" spans="1:4" ht="30" x14ac:dyDescent="0.25">
-      <c r="A17" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="B17" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="C17" s="2"/>
-    </row>
-    <row r="18" spans="1:4" ht="30" x14ac:dyDescent="0.25">
-      <c r="A18" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="B18" s="1" t="s">
-        <v>50</v>
       </c>
       <c r="C18" s="2"/>
     </row>
     <row r="19" spans="1:4" ht="45" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="B19" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="C19" s="2"/>
+    </row>
+    <row r="20" spans="1:4" ht="45" x14ac:dyDescent="0.25">
+      <c r="A20" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="B20" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="C20" s="2"/>
+    </row>
+    <row r="21" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+      <c r="A21" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="B21" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="C21" s="2"/>
+    </row>
+    <row r="22" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+      <c r="A22" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="B22" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="C22" s="2"/>
+    </row>
+    <row r="23" spans="1:4" ht="45" x14ac:dyDescent="0.25">
+      <c r="A23" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="B19" s="1" t="s">
+      <c r="B23" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="C19" s="2"/>
-      <c r="D19" s="5" t="s">
+      <c r="C23" s="2"/>
+      <c r="D23" s="5" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="20" spans="1:4" ht="60" x14ac:dyDescent="0.25">
-      <c r="A20" s="1" t="s">
+    <row r="24" spans="1:4" ht="60" x14ac:dyDescent="0.25">
+      <c r="A24" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="B20" s="1" t="s">
+      <c r="B24" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="C20" s="2"/>
-      <c r="D20" s="5" t="s">
+      <c r="C24" s="2"/>
+      <c r="D24" s="5" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A21" s="1" t="s">
+    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A25" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="B21" s="1" t="s">
+      <c r="B25" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="D21" s="1" t="s">
+      <c r="D25" s="1" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="22" spans="1:4" ht="45" x14ac:dyDescent="0.25">
-      <c r="A22" s="1" t="s">
+    <row r="26" spans="1:4" ht="45" x14ac:dyDescent="0.25">
+      <c r="A26" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="B22" s="1" t="s">
+      <c r="B26" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="D22" s="1" t="s">
+      <c r="D26" s="1" t="s">
         <v>57</v>
-      </c>
-    </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A23" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="B23" s="1" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A24" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="B24" s="1" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="25" spans="1:4" ht="30" x14ac:dyDescent="0.25">
-      <c r="A25" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="B25" s="1" t="s">
-        <v>60</v>
-      </c>
-      <c r="D25" s="1" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A26" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="B26" s="1" t="s">
-        <v>63</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A27" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="B27" s="1" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A28" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="B28" s="1" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+      <c r="A29" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="B29" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="D29" s="1" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A30" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="B30" s="1" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A31" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="B27" s="1" t="s">
+      <c r="B31" s="1" t="s">
         <v>62</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4" ht="45" x14ac:dyDescent="0.25">
+      <c r="A32" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="B32" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="D32" s="1" t="s">
+        <v>74</v>
       </c>
     </row>
   </sheetData>

</xml_diff>